<commit_message>
Add more personality models
</commit_message>
<xml_diff>
--- a/results/pooled_results_OR_multi_exposure_models_personality.xlsx
+++ b/results/pooled_results_OR_multi_exposure_models_personality.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Keiji\Documents\Research\ahs_fibromyalgia\results\Old\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Keiji\Documents\Research\ahs_fibromyalgia\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BB4870-EC30-49B9-A6B3-8E00E3C8B28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D9D972-8A67-4113-A0C8-82391E34218C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{797B858C-DA94-466A-A931-46BE830858D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="35">
   <si>
     <t>Depression</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>&lt;.0001</t>
+  </si>
+  <si>
+    <t>Depression + Hostility + Authority</t>
   </si>
 </sst>
 </file>
@@ -262,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -286,6 +289,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -632,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9215179F-2EFE-4E44-8C52-C38DCB1662E2}">
-  <dimension ref="B1:Q44"/>
+  <dimension ref="B1:V44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19" style="3" bestFit="1" customWidth="1"/>
@@ -641,9 +645,11 @@
     <col min="7" max="7" width="8.88671875" style="2"/>
     <col min="8" max="8" width="2.77734375" customWidth="1"/>
     <col min="13" max="13" width="2.77734375" customWidth="1"/>
+    <col min="18" max="18" width="2.77734375" customWidth="1"/>
+    <col min="22" max="22" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B1" s="5" t="s">
         <v>20</v>
       </c>
@@ -651,7 +657,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>22</v>
       </c>
@@ -659,37 +665,43 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="16" t="s">
+    <row r="4" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18"/>
-      <c r="I4" s="16" t="s">
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19"/>
+      <c r="I4" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18"/>
-      <c r="N4" s="16" t="s">
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="19"/>
+      <c r="N4" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="18"/>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="19"/>
+      <c r="S4" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="19"/>
+    </row>
+    <row r="5" spans="2:22" x14ac:dyDescent="0.3">
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
@@ -732,8 +744,21 @@
       <c r="Q6" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="R6" s="4"/>
+      <c r="S6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="T6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="U6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="V6" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>0</v>
       </c>
@@ -743,25 +768,32 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="15"/>
+      <c r="E7" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="16"/>
       <c r="G7" s="11"/>
       <c r="I7" s="1">
         <v>1</v>
       </c>
-      <c r="J7" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="15"/>
+      <c r="J7" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="16"/>
       <c r="L7" s="11"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="11"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S7" s="1">
+        <v>1</v>
+      </c>
+      <c r="T7" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U7" s="16"/>
+    </row>
+    <row r="8" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C8" s="6">
         <v>1</v>
       </c>
@@ -793,8 +825,20 @@
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="11"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S8" s="1">
+        <v>1.1069354</v>
+      </c>
+      <c r="T8" s="1">
+        <v>0.69061090000000003</v>
+      </c>
+      <c r="U8" s="1">
+        <v>1.7742347000000001</v>
+      </c>
+      <c r="V8" s="11">
+        <v>0.67276999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C9" s="6">
         <v>2</v>
       </c>
@@ -827,8 +871,20 @@
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="11"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S9" s="10">
+        <v>1.7951975</v>
+      </c>
+      <c r="T9" s="10">
+        <v>1.1134356999999999</v>
+      </c>
+      <c r="U9" s="10">
+        <v>2.8944052999999998</v>
+      </c>
+      <c r="V9" s="12">
+        <v>1.6369999999999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C10" s="6">
         <v>3</v>
       </c>
@@ -861,8 +917,20 @@
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="11"/>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S10" s="10">
+        <v>2.5909279000000001</v>
+      </c>
+      <c r="T10" s="10">
+        <v>1.4081748999999999</v>
+      </c>
+      <c r="U10" s="10">
+        <v>4.7670978000000002</v>
+      </c>
+      <c r="V10" s="12">
+        <v>2.2300000000000002E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C11" s="6"/>
       <c r="G11" s="11"/>
       <c r="I11" s="1"/>
@@ -873,8 +941,11 @@
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="11"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>17</v>
       </c>
@@ -884,10 +955,10 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="15"/>
+      <c r="E12" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="16"/>
       <c r="G12" s="11"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -896,13 +967,20 @@
       <c r="N12" s="1">
         <v>1</v>
       </c>
-      <c r="O12" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P12" s="15"/>
+      <c r="O12" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P12" s="16"/>
       <c r="Q12" s="11"/>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S12" s="1">
+        <v>1</v>
+      </c>
+      <c r="T12" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U12" s="16"/>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C13" s="6">
         <v>1</v>
       </c>
@@ -934,8 +1012,20 @@
       <c r="Q13" s="11">
         <v>7.5759999999999994E-2</v>
       </c>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S13" s="1">
+        <v>1.3838549</v>
+      </c>
+      <c r="T13" s="1">
+        <v>0.92239329999999997</v>
+      </c>
+      <c r="U13" s="1">
+        <v>2.0761799999999999</v>
+      </c>
+      <c r="V13" s="11">
+        <v>0.11645</v>
+      </c>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C14" s="6">
         <v>2</v>
       </c>
@@ -967,8 +1057,20 @@
       <c r="Q14" s="12">
         <v>3.3869999999999997E-2</v>
       </c>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S14" s="1">
+        <v>1.5123792</v>
+      </c>
+      <c r="T14" s="1">
+        <v>0.89909030000000001</v>
+      </c>
+      <c r="U14" s="1">
+        <v>2.5440057</v>
+      </c>
+      <c r="V14" s="11">
+        <v>0.11891</v>
+      </c>
+    </row>
+    <row r="15" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C15" s="6"/>
       <c r="G15" s="11"/>
       <c r="I15" s="1"/>
@@ -979,8 +1081,11 @@
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="11"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>18</v>
       </c>
@@ -991,21 +1096,28 @@
       <c r="I16" s="1">
         <v>1</v>
       </c>
-      <c r="J16" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K16" s="15"/>
+      <c r="J16" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16" s="16"/>
       <c r="L16" s="11"/>
       <c r="N16" s="1">
         <v>1</v>
       </c>
-      <c r="O16" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P16" s="15"/>
+      <c r="O16" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P16" s="16"/>
       <c r="Q16" s="11"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S16" s="1">
+        <v>1</v>
+      </c>
+      <c r="T16" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U16" s="16"/>
+    </row>
+    <row r="17" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C17" s="6">
         <v>1</v>
       </c>
@@ -1034,8 +1146,20 @@
       <c r="Q17" s="12">
         <v>4.861E-2</v>
       </c>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S17" s="1">
+        <v>1.6765410999999999</v>
+      </c>
+      <c r="T17" s="1">
+        <v>0.96339249999999998</v>
+      </c>
+      <c r="U17" s="1">
+        <v>2.9175960999999999</v>
+      </c>
+      <c r="V17" s="11">
+        <v>6.7519999999999997E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C18" s="6">
         <v>2</v>
       </c>
@@ -1065,8 +1189,21 @@
       <c r="Q18" s="12">
         <v>9.6500000000000006E-3</v>
       </c>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R18" s="3"/>
+      <c r="S18" s="10">
+        <v>1.8908403</v>
+      </c>
+      <c r="T18" s="10">
+        <v>1.0367629</v>
+      </c>
+      <c r="U18" s="10">
+        <v>3.4485000000000001</v>
+      </c>
+      <c r="V18" s="12">
+        <v>3.7749999999999999E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C19" s="6">
         <v>3</v>
       </c>
@@ -1095,8 +1232,20 @@
       <c r="Q19" s="12">
         <v>2.2610000000000002E-2</v>
       </c>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S19" s="1">
+        <v>2.0975494000000001</v>
+      </c>
+      <c r="T19" s="1">
+        <v>0.86529500000000004</v>
+      </c>
+      <c r="U19" s="1">
+        <v>5.0846396</v>
+      </c>
+      <c r="V19" s="11">
+        <v>0.10100000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C20" s="6"/>
       <c r="G20" s="11"/>
       <c r="I20" s="1"/>
@@ -1107,8 +1256,11 @@
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="11"/>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="1"/>
+    </row>
+    <row r="21" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1150,8 +1302,21 @@
       <c r="Q21" s="13" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R21" s="3"/>
+      <c r="S21" s="10">
+        <v>0.95204009999999994</v>
+      </c>
+      <c r="T21" s="10">
+        <v>0.93274380000000001</v>
+      </c>
+      <c r="U21" s="10">
+        <v>0.97173560000000003</v>
+      </c>
+      <c r="V21" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G22" s="11"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -1161,8 +1326,12 @@
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="11"/>
-    </row>
-    <row r="23" spans="2:17" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="S22" s="10"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="12"/>
+    </row>
+    <row r="23" spans="2:22" ht="16.2" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>24</v>
       </c>
@@ -1204,8 +1373,21 @@
       <c r="Q23" s="12">
         <v>2.7959999999999999E-2</v>
       </c>
-    </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R23" s="3"/>
+      <c r="S23" s="10">
+        <v>0.94097660000000005</v>
+      </c>
+      <c r="T23" s="10">
+        <v>0.89540609999999998</v>
+      </c>
+      <c r="U23" s="10">
+        <v>0.98886640000000003</v>
+      </c>
+      <c r="V23" s="12">
+        <v>1.635E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G24" s="11"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -1215,8 +1397,11 @@
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
       <c r="Q24" s="11"/>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+    </row>
+    <row r="25" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>6</v>
       </c>
@@ -1226,29 +1411,36 @@
       <c r="D25" s="1">
         <v>1</v>
       </c>
-      <c r="E25" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F25" s="15"/>
+      <c r="E25" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="16"/>
       <c r="G25" s="11"/>
       <c r="I25" s="1">
         <v>1</v>
       </c>
-      <c r="J25" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K25" s="15"/>
+      <c r="J25" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K25" s="16"/>
       <c r="L25" s="11"/>
       <c r="N25" s="1">
         <v>1</v>
       </c>
-      <c r="O25" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P25" s="15"/>
+      <c r="O25" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P25" s="16"/>
       <c r="Q25" s="11"/>
-    </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S25" s="1">
+        <v>1</v>
+      </c>
+      <c r="T25" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U25" s="16"/>
+    </row>
+    <row r="26" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C26" s="3" t="s">
         <v>1</v>
       </c>
@@ -1288,8 +1480,20 @@
       <c r="Q26" s="11">
         <v>0.18229000000000001</v>
       </c>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S26" s="1">
+        <v>1.4767136000000001</v>
+      </c>
+      <c r="T26" s="1">
+        <v>0.89306479999999999</v>
+      </c>
+      <c r="U26" s="1">
+        <v>2.4417970000000002</v>
+      </c>
+      <c r="V26" s="11">
+        <v>0.12866</v>
+      </c>
+    </row>
+    <row r="27" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C27" s="3" t="s">
         <v>2</v>
       </c>
@@ -1329,8 +1533,20 @@
       <c r="Q27" s="11">
         <v>0.20610000000000001</v>
       </c>
-    </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S27" s="1">
+        <v>1.6107001999999999</v>
+      </c>
+      <c r="T27" s="1">
+        <v>0.90319280000000002</v>
+      </c>
+      <c r="U27" s="1">
+        <v>2.8724267999999999</v>
+      </c>
+      <c r="V27" s="11">
+        <v>0.10628</v>
+      </c>
+    </row>
+    <row r="28" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G28" s="11"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
@@ -1340,8 +1556,11 @@
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="11"/>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+    </row>
+    <row r="29" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>7</v>
       </c>
@@ -1351,29 +1570,36 @@
       <c r="D29" s="1">
         <v>1</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F29" s="15"/>
+      <c r="E29" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="16"/>
       <c r="G29" s="11"/>
       <c r="I29" s="1">
         <v>1</v>
       </c>
-      <c r="J29" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K29" s="15"/>
+      <c r="J29" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K29" s="16"/>
       <c r="L29" s="11"/>
       <c r="N29" s="1">
         <v>1</v>
       </c>
-      <c r="O29" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P29" s="15"/>
+      <c r="O29" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P29" s="16"/>
       <c r="Q29" s="11"/>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S29" s="1">
+        <v>1</v>
+      </c>
+      <c r="T29" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U29" s="16"/>
+    </row>
+    <row r="30" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C30" s="3" t="s">
         <v>4</v>
       </c>
@@ -1413,8 +1639,20 @@
       <c r="Q30" s="11">
         <v>0.18969</v>
       </c>
-    </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S30" s="1">
+        <v>0.7425235</v>
+      </c>
+      <c r="T30" s="1">
+        <v>0.51006649999999998</v>
+      </c>
+      <c r="U30" s="1">
+        <v>1.0809200999999999</v>
+      </c>
+      <c r="V30" s="11">
+        <v>0.12018</v>
+      </c>
+    </row>
+    <row r="31" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G31" s="11"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
@@ -1424,8 +1662,11 @@
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
       <c r="Q31" s="11"/>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+    </row>
+    <row r="32" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>8</v>
       </c>
@@ -1435,29 +1676,36 @@
       <c r="D32" s="1">
         <v>1</v>
       </c>
-      <c r="E32" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F32" s="15"/>
+      <c r="E32" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" s="16"/>
       <c r="G32" s="11"/>
       <c r="I32" s="1">
         <v>1</v>
       </c>
-      <c r="J32" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K32" s="15"/>
+      <c r="J32" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K32" s="16"/>
       <c r="L32" s="11"/>
       <c r="N32" s="1">
         <v>1</v>
       </c>
-      <c r="O32" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P32" s="15"/>
+      <c r="O32" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P32" s="16"/>
       <c r="Q32" s="11"/>
-    </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S32" s="1">
+        <v>1</v>
+      </c>
+      <c r="T32" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U32" s="16"/>
+    </row>
+    <row r="33" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C33" s="3" t="s">
         <v>10</v>
       </c>
@@ -1497,8 +1745,20 @@
       <c r="Q33" s="11">
         <v>0.88415999999999995</v>
       </c>
-    </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S33" s="1">
+        <v>1.1313055999999999</v>
+      </c>
+      <c r="T33" s="1">
+        <v>0.51853939999999998</v>
+      </c>
+      <c r="U33" s="1">
+        <v>2.4681872999999999</v>
+      </c>
+      <c r="V33" s="11">
+        <v>0.75651999999999997</v>
+      </c>
+    </row>
+    <row r="34" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C34" s="3" t="s">
         <v>11</v>
       </c>
@@ -1538,8 +1798,20 @@
       <c r="Q34" s="11">
         <v>0.36929000000000001</v>
       </c>
-    </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S34" s="1">
+        <v>1.4673392000000001</v>
+      </c>
+      <c r="T34" s="1">
+        <v>0.57508139999999996</v>
+      </c>
+      <c r="U34" s="1">
+        <v>3.7439643999999999</v>
+      </c>
+      <c r="V34" s="11">
+        <v>0.42224</v>
+      </c>
+    </row>
+    <row r="35" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G35" s="11"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
@@ -1549,8 +1821,11 @@
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="11"/>
-    </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S35" s="1"/>
+      <c r="T35" s="1"/>
+      <c r="U35" s="1"/>
+    </row>
+    <row r="36" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>25</v>
       </c>
@@ -1560,29 +1835,36 @@
       <c r="D36" s="1">
         <v>1</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" s="15"/>
+      <c r="E36" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" s="16"/>
       <c r="G36" s="11"/>
       <c r="I36" s="1">
         <v>1</v>
       </c>
-      <c r="J36" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K36" s="15"/>
+      <c r="J36" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="16"/>
       <c r="L36" s="11"/>
       <c r="N36" s="1">
         <v>1</v>
       </c>
-      <c r="O36" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P36" s="15"/>
+      <c r="O36" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P36" s="16"/>
       <c r="Q36" s="11"/>
-    </row>
-    <row r="37" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S36" s="1">
+        <v>1</v>
+      </c>
+      <c r="T36" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U36" s="16"/>
+    </row>
+    <row r="37" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C37" s="3" t="s">
         <v>27</v>
       </c>
@@ -1624,8 +1906,21 @@
       <c r="Q37" s="12">
         <v>1.34E-3</v>
       </c>
-    </row>
-    <row r="38" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="R37" s="3"/>
+      <c r="S37" s="10">
+        <v>2.2084725999999999</v>
+      </c>
+      <c r="T37" s="10">
+        <v>1.3558211</v>
+      </c>
+      <c r="U37" s="10">
+        <v>3.5973413999999999</v>
+      </c>
+      <c r="V37" s="12">
+        <v>1.47E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G38" s="11"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
@@ -1635,8 +1930,11 @@
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
       <c r="Q38" s="11"/>
-    </row>
-    <row r="39" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S38" s="1"/>
+      <c r="T38" s="1"/>
+      <c r="U38" s="1"/>
+    </row>
+    <row r="39" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>28</v>
       </c>
@@ -1646,29 +1944,36 @@
       <c r="D39" s="1">
         <v>1</v>
       </c>
-      <c r="E39" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" s="15"/>
+      <c r="E39" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F39" s="16"/>
       <c r="G39" s="11"/>
       <c r="I39" s="1">
         <v>1</v>
       </c>
-      <c r="J39" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K39" s="15"/>
+      <c r="J39" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K39" s="16"/>
       <c r="L39" s="11"/>
       <c r="N39" s="1">
         <v>1</v>
       </c>
-      <c r="O39" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P39" s="15"/>
+      <c r="O39" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P39" s="16"/>
       <c r="Q39" s="11"/>
-    </row>
-    <row r="40" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S39" s="1">
+        <v>1</v>
+      </c>
+      <c r="T39" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U39" s="16"/>
+    </row>
+    <row r="40" spans="2:22" x14ac:dyDescent="0.3">
       <c r="C40" s="3" t="s">
         <v>4</v>
       </c>
@@ -1708,8 +2013,20 @@
       <c r="Q40" s="11">
         <v>5.364E-2</v>
       </c>
-    </row>
-    <row r="41" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S40" s="1">
+        <v>1.6385312999999999</v>
+      </c>
+      <c r="T40" s="1">
+        <v>0.93709330000000002</v>
+      </c>
+      <c r="U40" s="1">
+        <v>2.8650131999999999</v>
+      </c>
+      <c r="V40" s="11">
+        <v>8.3229999999999998E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:22" x14ac:dyDescent="0.3">
       <c r="G41" s="11"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
@@ -1719,8 +2036,11 @@
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
       <c r="Q41" s="11"/>
-    </row>
-    <row r="42" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="S41" s="1"/>
+      <c r="T41" s="1"/>
+      <c r="U41" s="1"/>
+    </row>
+    <row r="42" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>29</v>
       </c>
@@ -1730,29 +2050,36 @@
       <c r="D42" s="1">
         <v>1</v>
       </c>
-      <c r="E42" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F42" s="15"/>
+      <c r="E42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F42" s="16"/>
       <c r="G42" s="11"/>
       <c r="I42" s="1">
         <v>1</v>
       </c>
-      <c r="J42" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K42" s="15"/>
+      <c r="J42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K42" s="16"/>
       <c r="L42" s="11"/>
       <c r="N42" s="1">
         <v>1</v>
       </c>
-      <c r="O42" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="P42" s="15"/>
+      <c r="O42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P42" s="16"/>
       <c r="Q42" s="11"/>
-    </row>
-    <row r="43" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="S42" s="1">
+        <v>1</v>
+      </c>
+      <c r="T42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U42" s="16"/>
+    </row>
+    <row r="43" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="4"/>
       <c r="C43" s="4" t="s">
         <v>4</v>
@@ -1795,10 +2122,23 @@
       <c r="Q43" s="14" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="44" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="8">
+        <v>3.0591674000000002</v>
+      </c>
+      <c r="T43" s="8">
+        <v>1.9761858000000001</v>
+      </c>
+      <c r="U43" s="8">
+        <v>4.7356404000000003</v>
+      </c>
+      <c r="V43" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="37">
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="J42:K42"/>
     <mergeCell ref="O42:P42"/>
@@ -1826,6 +2166,16 @@
     <mergeCell ref="J29:K29"/>
     <mergeCell ref="O25:P25"/>
     <mergeCell ref="O29:P29"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="T12:U12"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="T32:U32"/>
+    <mergeCell ref="T36:U36"/>
+    <mergeCell ref="T39:U39"/>
+    <mergeCell ref="T42:U42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>